<commit_message>
fix: shorten metro branch and rebalance outer route
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M3候选.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M3候选.xlsx
@@ -694,7 +694,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 河坊街铺</t>
+          <t xml:space="preserve">47 滨江国际社区</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9 钱塘潮</t>
+          <t xml:space="preserve">39 钱江新城</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">14 项目验收</t>
+          <t xml:space="preserve">42 地铁补给站</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">19 人才事件</t>
+          <t xml:space="preserve">48 大运河艺术馆</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25 杭城事件</t>
+          <t xml:space="preserve">43 未来路演厅</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">47 滨江国际社区</t>
+          <t xml:space="preserve">40 地铁快线</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40 地铁快线</t>
+          <t xml:space="preserve">9 钱塘潮</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">42 地铁补给站</t>
+          <t xml:space="preserve">44 未来科技城</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">48 大运河艺术馆</t>
+          <t xml:space="preserve">14 项目验收</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">44 未来科技城</t>
+          <t xml:space="preserve">25 杭城事件</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">39 钱江新城</t>
+          <t xml:space="preserve">3 河坊街铺</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">43 未来路演厅</t>
+          <t xml:space="preserve">19 人才事件</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E22" s="2">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E25" s="2">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E26" s="2">

</xml_diff>

<commit_message>
fix: balance metro branch density and curvature
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M3候选.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M3候选.xlsx
@@ -948,7 +948,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">39 钱江新城</t>
+          <t xml:space="preserve">9 钱塘潮</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">48 大运河艺术馆</t>
+          <t xml:space="preserve">19 人才事件</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40 地铁快线</t>
+          <t xml:space="preserve">48 大运河艺术馆</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9 钱塘潮</t>
+          <t xml:space="preserve">40 地铁快线</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">19 人才事件</t>
+          <t xml:space="preserve">39 钱江新城</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">外环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="E26" s="2">

</xml_diff>

<commit_message>
fix: balance both branch routes together
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M3候选.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M3候选.xlsx
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">31 水上巴士</t>
+          <t xml:space="preserve">40 地铁快线</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">地铁快线内环</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35 运河灯会</t>
+          <t xml:space="preserve">44 未来科技城</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40 地铁快线</t>
+          <t xml:space="preserve">30 香积寺晨市</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">44 未来科技城</t>
+          <t xml:space="preserve">34 拱宸桥码头</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 香积寺晨市</t>
+          <t xml:space="preserve">31 水上巴士</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">34 拱宸桥码头</t>
+          <t xml:space="preserve">35 运河灯会</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: move shortcut nodes onto main route
Co-authored-by: TRAE CLI <traecli@bytedance.com>
</commit_message>
<xml_diff>
--- a/docs/design/杭城合伙局-数值设计-M3候选.xlsx
+++ b/docs/design/杭城合伙局-数值设计-M3候选.xlsx
@@ -612,7 +612,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 龙井茶园</t>
+          <t xml:space="preserve">34 拱宸桥码头</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 杭城事件</t>
+          <t xml:space="preserve">32 运河事件</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9 钱塘潮</t>
+          <t xml:space="preserve">46 运河运动公园</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 良渚陶艺村</t>
+          <t xml:space="preserve">35 运河灯会</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20 西溪营地</t>
+          <t xml:space="preserve">30 香积寺晨市</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">27 道具补给站</t>
+          <t xml:space="preserve">40 地铁快线</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40 地铁快线</t>
+          <t xml:space="preserve">20 西溪营地</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">32 运河事件</t>
+          <t xml:space="preserve">33 桥西文创园</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">33 桥西文创园</t>
+          <t xml:space="preserve">6 杭城事件</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">46 运河运动公园</t>
+          <t xml:space="preserve">36 西湖接驳</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">44 未来科技城</t>
+          <t xml:space="preserve">1 龙井茶园</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">36 西湖接驳</t>
+          <t xml:space="preserve">16 良渚陶艺村</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 香积寺晨市</t>
+          <t xml:space="preserve">41 文三数字街</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">地铁快线内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">41 文三数字街</t>
+          <t xml:space="preserve">27 道具补给站</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">34 拱宸桥码头</t>
+          <t xml:space="preserve">44 未来科技城</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">35 运河灯会</t>
+          <t xml:space="preserve">9 钱塘潮</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">水上巴士内环</t>
+          <t xml:space="preserve">外环</t>
         </is>
       </c>
       <c r="E24" s="2">

</xml_diff>